<commit_message>
Añadimos modulos al form
</commit_message>
<xml_diff>
--- a/SmartMoney_Screener.xlsx
+++ b/SmartMoney_Screener.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,23 +476,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>tsla</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>427.85</v>
+        <v>449.31</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>VENTA</t>
+          <t>COMPRA FUERTE</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -516,11 +516,266 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.67</v>
+        <v>0.4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-12 19:59</t>
+          <t>2026-05-14 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1006.34</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>65</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>235.29</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GOOG</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>396.06</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>298.17</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>65</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>COST</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1034.25</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>65</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-05-14 18:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se cambia la ventana E_Ticker para que sea eitable
</commit_message>
<xml_diff>
--- a/SmartMoney_Screener.xlsx
+++ b/SmartMoney_Screener.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,11 +476,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>449.31</v>
+        <v>228.52</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.4</v>
+        <v>0.58</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1006.34</v>
+        <v>432.25</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -567,22 +567,22 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>235.29</v>
+        <v>440.04</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,26 +614,26 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NEUTRO</t>
+          <t>ACUMULANDO</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.68</v>
+        <v>1.08</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>396.06</v>
+        <v>286.31</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -669,22 +669,22 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.37</v>
+        <v>0.54</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>298.17</v>
+        <v>1833.98</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -720,22 +720,22 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.34</v>
+        <v>0.4</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1034.25</v>
+        <v>735.8200000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -771,11 +771,62 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.29</v>
+        <v>0.65</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-05-14 18:43</t>
+          <t>2026-05-15 18:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>117.04</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-05-15 18:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Limpiamos ventanas de texto cuando analizamos Ticker
</commit_message>
<xml_diff>
--- a/SmartMoney_Screener.xlsx
+++ b/SmartMoney_Screener.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,11 +476,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>228.52</v>
+        <v>1002.03</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -516,22 +516,22 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.58</v>
+        <v>0.35</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2026-05-15 18:47</t>
+          <t>2026-05-15 18:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>432.25</v>
+        <v>228.06</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -567,22 +567,22 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.4</v>
+        <v>0.59</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2026-05-15 18:47</t>
+          <t>2026-05-15 18:58</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>440.04</v>
+        <v>392.36</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,26 +614,26 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ACUMULANDO</t>
+          <t>NEUTRO</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1.08</v>
+        <v>0.43</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2026-05-15 18:47</t>
+          <t>2026-05-15 18:58</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>286.31</v>
+        <v>302.58</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -669,22 +669,22 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.54</v>
+        <v>0.59</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-05-15 18:47</t>
+          <t>2026-05-15 18:58</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>COST</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1833.98</v>
+        <v>1046.32</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -720,113 +720,11 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.4</v>
+        <v>0.54</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2026-05-15 18:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>735.8200000000001</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>COMPRA FUERTE</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>65</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>DEBIL</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>COMPRANDO</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>NEUTRO</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2026-05-15 18:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>CSCO</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>117.04</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>COMPRA FUERTE</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>65</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>FUERTE</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>DEBIL</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>COMPRANDO</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>NEUTRO</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>2026-05-15 18:47</t>
+          <t>2026-05-15 18:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
modificamos el tamaño de las columnas
</commit_message>
<xml_diff>
--- a/SmartMoney_Screener.xlsx
+++ b/SmartMoney_Screener.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,11 +476,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LLY</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1018.87</v>
+        <v>233</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -488,39 +488,1110 @@
         </is>
       </c>
       <c r="D2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>274</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>65</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>FUERTE</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>DEBIL</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>COMPRANDO</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>NEUTRO</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-05-21 12:46</t>
+      <c r="J3" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>518.09</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>65</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>449.68</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>923.52</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>COMPRA FUERTE</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>65</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IONQ</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>70.14</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>55</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RGTI</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>27.03</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>55</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>QUBT</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>12.24</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>COMPRA TEMPRANA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>QBTS</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>29.49</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>55</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IBM</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>264.22</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>55</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>426.99</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>55</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>204.83</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>55</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>ACUMULANDO</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ARQQ</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>16.91</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>COMPRA TEMPRANA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>120.89</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>COMPRA TEMPRANA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>318</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1927.63</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>40</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>RTX</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>178.96</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ESPERA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>40</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>COMPRANDO</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>390.13</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>25</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>VENDIENDO</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>214.25</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>VENDIENDO</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>373.85</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>25</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FUERTE</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>VENDIENDO</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CSCO</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>118.64</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>VENDIENDO</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>NEUTRO</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>480.64</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>VENTA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>DEBIL</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>VENDIENDO</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DISTRIBUYENDO</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:20</t>
         </is>
       </c>
     </row>

</xml_diff>